<commit_message>
cambios trabajador en puesto
</commit_message>
<xml_diff>
--- a/assets/docs/empleado/actualizar/empleado.xlsx
+++ b/assets/docs/empleado/actualizar/empleado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\cnomina\assets\docs\empleado\actualizar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C3D6855-13FE-49C2-BE6F-F2D475B08F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DF0A0E2-8C0A-449A-A3E5-9D9E812AD4BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{65C88286-55CE-464B-A52D-D9951CA36E83}"/>
+    <workbookView xWindow="-108" yWindow="252" windowWidth="23256" windowHeight="11952" xr2:uid="{65C88286-55CE-464B-A52D-D9951CA36E83}"/>
   </bookViews>
   <sheets>
     <sheet name="Empleados" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t># EMPLEADO</t>
   </si>
@@ -55,9 +55,6 @@
     <t>RFC</t>
   </si>
   <si>
-    <t>TIPO DE TRABAJADOR</t>
-  </si>
-  <si>
     <t>CUENTA BANCARIA</t>
   </si>
   <si>
@@ -80,9 +77,6 @@
   </si>
   <si>
     <t>XXXXXXXXXXXXX</t>
-  </si>
-  <si>
-    <t>BASE</t>
   </si>
   <si>
     <t>CATORCENAL</t>
@@ -474,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F527379-0796-45E5-B8DA-938739265192}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.21875" style="4" bestFit="1" customWidth="1"/>
@@ -483,16 +477,15 @@
     <col min="4" max="4" width="17.44140625" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="17.44140625" style="3" customWidth="1"/>
     <col min="7" max="7" width="19" style="4" customWidth="1"/>
-    <col min="8" max="8" width="16.44140625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="21.77734375" style="3" customWidth="1"/>
     <col min="9" max="9" width="19.77734375" style="3" customWidth="1"/>
-    <col min="10" max="10" width="18.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.5546875" style="3"/>
+    <col min="10" max="10" width="22.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="11.5546875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -506,10 +499,10 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>4</v>
@@ -529,49 +522,43 @@
       <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>15</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>16</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>